<commit_message>
Day 02 (14-Aug-2026): Practice 02 Swap Two Numbers & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -700,7 +700,60 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1"/>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>14-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>430</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>945</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>495</v>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N7" s="10" t="inlineStr">
+        <is>
+          <t>Day 02: 02_swap_two_numbers.py (Swap Numbers without 3rd Var) | Swapped two variables using arithmetic addition and subtraction.</t>
+        </is>
+      </c>
+    </row>
     <row r="8" ht="22" customHeight="1"/>
     <row r="9" ht="22" customHeight="1"/>
     <row r="10" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 03 (15-Aug-2026): Practice 03 Data Type Identifier & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -754,7 +754,60 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1"/>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>15-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>440</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>110</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>140</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>880</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>560</v>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
+          <t>Day 03: 03_data_type_identifier.py (Identify Data Types) | Checked variable types using type().__name__ built-in function.</t>
+        </is>
+      </c>
+    </row>
     <row r="9" ht="22" customHeight="1"/>
     <row r="10" ht="22" customHeight="1"/>
     <row r="11" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 04 (16-Aug-2026): Practice 04 Even Or Odd & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -808,7 +808,60 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1"/>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>16-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>460</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>170</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>950</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>490</v>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>Day 04: 04_even_or_odd.py (Check Even or Odd Number) | Checked parity of integer using modulo operator (% 2).</t>
+        </is>
+      </c>
+    </row>
     <row r="10" ht="22" customHeight="1"/>
     <row r="11" ht="22" customHeight="1"/>
     <row r="12" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 05 (17-Aug-2026): Practice 05 Greatest Of Two & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -862,7 +862,60 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1"/>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>17-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>470</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>110</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>140</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>1005</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>435</v>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>Day 05: 05_greatest_of_two.py (Greatest of Two Numbers) | Compared two variables using relational conditions.</t>
+        </is>
+      </c>
+    </row>
     <row r="11" ht="22" customHeight="1"/>
     <row r="12" ht="22" customHeight="1"/>
     <row r="13" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 06 (18-Aug-2026): Practice 06 Simple Interest & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -916,7 +916,60 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1"/>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>18-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>430</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>110</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>930</v>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>510</v>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M11" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>Day 06: 06_simple_interest.py (Calculate Simple Interest) | Computed simple interest and maturity amount from P, R, T.</t>
+        </is>
+      </c>
+    </row>
     <row r="12" ht="22" customHeight="1"/>
     <row r="13" ht="22" customHeight="1"/>
     <row r="14" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 07 (19-Aug-2026): Practice 07 Secure Login Display & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -970,7 +970,60 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1"/>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>19-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>440</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>105</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>135</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>160</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>875</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>565</v>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N12" s="7" t="inlineStr">
+        <is>
+          <t>Day 07: 07_secure_login_display.py (Masked Password Display) | Accepted username and password, masked output with asterisks.</t>
+        </is>
+      </c>
+    </row>
     <row r="13" ht="22" customHeight="1"/>
     <row r="14" ht="22" customHeight="1"/>
     <row r="15" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 08 (20-Aug-2026): Practice 08 Sum Of Two Numbers & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1024,7 +1024,60 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1"/>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>20-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>435</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>155</v>
+      </c>
+      <c r="I13" s="9" t="n">
+        <v>910</v>
+      </c>
+      <c r="J13" s="9" t="n">
+        <v>530</v>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M13" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N13" s="10" t="inlineStr">
+        <is>
+          <t>Day 08: 08_sum_of_two_numbers.py (Sum of Two Numbers) | Computed sum of float numbers with formatted display.</t>
+        </is>
+      </c>
+    </row>
     <row r="14" ht="22" customHeight="1"/>
     <row r="15" ht="22" customHeight="1"/>
     <row r="16" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 09 (21-Aug-2026): Practice 09 Positive Negative Zero & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1078,7 +1078,60 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1"/>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>21-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>430</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>110</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>140</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>155</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>970</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>470</v>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>Day 09: 09_positive_negative_zero.py (Number Classification) | Classified integers as positive, negative or zero.</t>
+        </is>
+      </c>
+    </row>
     <row r="15" ht="22" customHeight="1"/>
     <row r="16" ht="22" customHeight="1"/>
     <row r="17" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 10 (22-Aug-2026): Practice 10 Leap Year & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1132,7 +1132,60 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1"/>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>22-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>420</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>160</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="I15" s="9" t="n">
+        <v>880</v>
+      </c>
+      <c r="J15" s="9" t="n">
+        <v>560</v>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M15" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N15" s="10" t="inlineStr">
+        <is>
+          <t>Day 10: 10_leap_year.py (Check Leap Year Conditions) | Evaluated 400, 100, and 4 divisibility rules for leap years.</t>
+        </is>
+      </c>
+    </row>
     <row r="16" ht="22" customHeight="1"/>
     <row r="17" ht="22" customHeight="1"/>
     <row r="18" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 11 (23-Aug-2026): Practice 11 Grade Calculator & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1186,7 +1186,60 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1"/>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>23-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>460</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>130</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>970</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>470</v>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N16" s="7" t="inlineStr">
+        <is>
+          <t>Day 11: 11_grade_calculator.py (Grades using if-elif-else) | Assigned academic letter grades (A+, A, B, C, F) based on marks.</t>
+        </is>
+      </c>
+    </row>
     <row r="17" ht="22" customHeight="1"/>
     <row r="18" ht="22" customHeight="1"/>
     <row r="19" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 12 (24-Aug-2026): Practice 12 Print 1 To 10 & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1240,7 +1240,60 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1"/>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>24-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>470</v>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>140</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>165</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="9" t="n">
+        <v>165</v>
+      </c>
+      <c r="I17" s="9" t="n">
+        <v>1045</v>
+      </c>
+      <c r="J17" s="9" t="n">
+        <v>395</v>
+      </c>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M17" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N17" s="10" t="inlineStr">
+        <is>
+          <t>Day 12: 12_print_1_to_10.py (Print Numbers 1 to 10) | Iterated numbers 1 to 10 on a single line using for loop.</t>
+        </is>
+      </c>
+    </row>
     <row r="18" ht="22" customHeight="1"/>
     <row r="19" ht="22" customHeight="1"/>
     <row r="20" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 13 (25-Aug-2026): Practice 13 Even Numbers 1 To 50 & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1294,7 +1294,60 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1"/>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>25-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>430</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>105</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>145</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>920</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>520</v>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>Day 13: 13_even_numbers_1_to_50.py (Even Numbers 1 to 50) | Generated even numbers sequence using range(2, 51, 2).</t>
+        </is>
+      </c>
+    </row>
     <row r="19" ht="22" customHeight="1"/>
     <row r="20" ht="22" customHeight="1"/>
     <row r="21" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 14 (26-Aug-2026): Practice 14 Multiplication Table & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1348,7 +1348,60 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1"/>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>26-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>435</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>115</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>155</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="I19" s="9" t="n">
+        <v>890</v>
+      </c>
+      <c r="J19" s="9" t="n">
+        <v>550</v>
+      </c>
+      <c r="K19" s="8" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L19" s="8" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M19" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N19" s="10" t="inlineStr">
+        <is>
+          <t>Day 14: 14_multiplication_table.py (Multiplication Table) | Formatted multiplication table from 1 to 10 for any number.</t>
+        </is>
+      </c>
+    </row>
     <row r="20" ht="22" customHeight="1"/>
     <row r="21" ht="22" customHeight="1"/>
     <row r="22" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 15 (27-Aug-2026): Practice 15 Count Digits & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1402,7 +1402,60 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1"/>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>27-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>435</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>110</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>930</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>510</v>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>Day 15: 15_count_digits.py (Count Digits of a Number) | Counted total number of digits in large integers.</t>
+        </is>
+      </c>
+    </row>
     <row r="21" ht="22" customHeight="1"/>
     <row r="22" ht="22" customHeight="1"/>
     <row r="23" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 16 (28-Aug-2026): Practice 16 Factorial Function & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1456,7 +1456,60 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1"/>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>28-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>430</v>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>140</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="I21" s="9" t="n">
+        <v>960</v>
+      </c>
+      <c r="J21" s="9" t="n">
+        <v>480</v>
+      </c>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M21" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N21" s="10" t="inlineStr">
+        <is>
+          <t>Day 16: 16_factorial_function.py (Factorial Function) | Defined find_factorial(n) function returning product.</t>
+        </is>
+      </c>
+    </row>
     <row r="22" ht="22" customHeight="1"/>
     <row r="23" ht="22" customHeight="1"/>
     <row r="24" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 17 (29-Aug-2026): Practice 17 Prime Check Function & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1510,7 +1510,60 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1"/>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>29-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>425</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>110</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>160</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>880</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>560</v>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N22" s="7" t="inlineStr">
+        <is>
+          <t>Day 17: 17_prime_check_function.py (Function to Check Prime) | Created is_prime(n) function with square root boundary.</t>
+        </is>
+      </c>
+    </row>
     <row r="23" ht="22" customHeight="1"/>
     <row r="24" ht="22" customHeight="1"/>
     <row r="25" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 18 (30-Aug-2026): Practice 18 Reverse String Function & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1564,7 +1564,60 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1"/>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>30-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="n">
+        <v>435</v>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>105</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>145</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>155</v>
+      </c>
+      <c r="I23" s="9" t="n">
+        <v>880</v>
+      </c>
+      <c r="J23" s="9" t="n">
+        <v>560</v>
+      </c>
+      <c r="K23" s="8" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L23" s="8" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M23" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N23" s="10" t="inlineStr">
+        <is>
+          <t>Day 18: 18_reverse_string_function.py (Reverse String Function) | Wrote reverse_string(text) function returning text[::-1].</t>
+        </is>
+      </c>
+    </row>
     <row r="24" ht="22" customHeight="1"/>
     <row r="25" ht="22" customHeight="1"/>
     <row r="26" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 19 (31-Aug-2026): Practice 19 Fizz Buzz & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1618,7 +1618,60 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1"/>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>31-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>460</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>125</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>1010</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>430</v>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N24" s="7" t="inlineStr">
+        <is>
+          <t>Day 19: 19_fizz_buzz.py (FizzBuzz 1 to 50) | Printed Fizz, Buzz, and FizzBuzz for multiples of 3 and 5.</t>
+        </is>
+      </c>
+    </row>
     <row r="25" ht="22" customHeight="1"/>
     <row r="26" ht="22" customHeight="1"/>
     <row r="27" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 20 (01-Sep-2026): Practice 20 Pos Neg Zero Counter & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1672,7 +1672,60 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1"/>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>01-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="n">
+        <v>465</v>
+      </c>
+      <c r="C25" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>160</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>180</v>
+      </c>
+      <c r="I25" s="9" t="n">
+        <v>1030</v>
+      </c>
+      <c r="J25" s="9" t="n">
+        <v>410</v>
+      </c>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L25" s="8" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M25" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N25" s="10" t="inlineStr">
+        <is>
+          <t>Day 20: 20_pos_neg_zero_counter.py (Count Pos, Neg, Zeros) | Iterated through array and counted positive, negative, zero values.</t>
+        </is>
+      </c>
+    </row>
     <row r="26" ht="22" customHeight="1"/>
     <row r="27" ht="22" customHeight="1"/>
     <row r="28" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 21 (02-Sep-2026): Practice 21 Even Odd Sums & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1726,7 +1726,60 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="22" customHeight="1"/>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>02-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>430</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>165</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>900</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>540</v>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N26" s="7" t="inlineStr">
+        <is>
+          <t>Day 21: 21_even_odd_sums.py (Separate Sum of Even and Odd) | Calculated separate sum of evens and sum of odds up to N.</t>
+        </is>
+      </c>
+    </row>
     <row r="27" ht="22" customHeight="1"/>
     <row r="28" ht="22" customHeight="1"/>
     <row r="29" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 22 (03-Sep-2026): Practice 22 Custom Multiplication Table & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1780,7 +1780,60 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="22" customHeight="1"/>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>03-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>430</v>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>110</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="I27" s="9" t="n">
+        <v>930</v>
+      </c>
+      <c r="J27" s="9" t="n">
+        <v>510</v>
+      </c>
+      <c r="K27" s="8" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L27" s="8" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M27" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N27" s="10" t="inlineStr">
+        <is>
+          <t>Day 22: 22_custom_multiplication_table.py (Custom Range Table) | Generated multiplication table between custom multiplier limits.</t>
+        </is>
+      </c>
+    </row>
     <row r="28" ht="22" customHeight="1"/>
     <row r="29" ht="22" customHeight="1"/>
     <row r="30" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 23 (04-Sep-2026): Practice 23 Largest Without Max & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1834,7 +1834,60 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1"/>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>04-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="n">
+        <v>435</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>110</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>980</v>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>460</v>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N28" s="7" t="inlineStr">
+        <is>
+          <t>Day 23: 23_largest_without_max.py (Find Largest without max()) | Found maximum number in array without using max() built-in.</t>
+        </is>
+      </c>
+    </row>
     <row r="29" ht="22" customHeight="1"/>
     <row r="30" ht="22" customHeight="1"/>
     <row r="31" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 24 (05-Sep-2026): Practice 24 Largest And Smallest & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1888,7 +1888,60 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="22" customHeight="1"/>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>05-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="n">
+        <v>425</v>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>115</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>155</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="I29" s="9" t="n">
+        <v>880</v>
+      </c>
+      <c r="J29" s="9" t="n">
+        <v>560</v>
+      </c>
+      <c r="K29" s="8" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L29" s="8" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M29" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N29" s="10" t="inlineStr">
+        <is>
+          <t>Day 24: 24_largest_and_smallest.py (Largest &amp; Smallest) | Tracked both smallest and largest elements in one loop.</t>
+        </is>
+      </c>
+    </row>
     <row r="30" ht="22" customHeight="1"/>
     <row r="31" ht="22" customHeight="1"/>
     <row r="32" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 25 (06-Sep-2026): Practice 25 Reverse And Palindrome Number & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1942,7 +1942,60 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="22" customHeight="1"/>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>06-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="n">
+        <v>430</v>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>160</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>900</v>
+      </c>
+      <c r="J30" s="6" t="n">
+        <v>540</v>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M30" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N30" s="7" t="inlineStr">
+        <is>
+          <t>Day 25: 25_reverse_and_palindrome_number.py (Palindrome Number) | Reversed digits using % 10 and checked palindrome equality.</t>
+        </is>
+      </c>
+    </row>
     <row r="31" ht="22" customHeight="1"/>
     <row r="32" ht="22" customHeight="1"/>
     <row r="33" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 26 (07-Sep-2026): Practice 26 Sum Of Digits Analysis & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1996,7 +1996,60 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="22" customHeight="1"/>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>07-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="n">
+        <v>460</v>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>170</v>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="9" t="n">
+        <v>170</v>
+      </c>
+      <c r="I31" s="9" t="n">
+        <v>1030</v>
+      </c>
+      <c r="J31" s="9" t="n">
+        <v>410</v>
+      </c>
+      <c r="K31" s="8" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L31" s="8" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M31" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N31" s="10" t="inlineStr">
+        <is>
+          <t>Day 26: 26_sum_of_digits_analysis.py (Sum of Digits Analysis) | Calculated digit sum and verified divisibility by 3 and 9.</t>
+        </is>
+      </c>
+    </row>
     <row r="32" ht="22" customHeight="1"/>
     <row r="33" ht="22" customHeight="1"/>
     <row r="34" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 27 (08-Sep-2026): Practice 27 Prime Numbers In Range & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2050,7 +2050,60 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="22" customHeight="1"/>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>08-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>465</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>125</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>145</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>170</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>1010</v>
+      </c>
+      <c r="J32" s="6" t="n">
+        <v>430</v>
+      </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M32" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N32" s="7" t="inlineStr">
+        <is>
+          <t>Day 27: 27_prime_numbers_in_range.py (Primes 1 to N No Funcs) | Printed all primes in 1 to N range using nested loops.</t>
+        </is>
+      </c>
+    </row>
     <row r="33" ht="22" customHeight="1"/>
     <row r="34" ht="22" customHeight="1"/>
     <row r="35" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 28 (09-Sep-2026): Practice 28 Prime Factors & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2104,7 +2104,60 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="22" customHeight="1"/>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>09-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="n">
+        <v>435</v>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>110</v>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="F33" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="9" t="n">
+        <v>155</v>
+      </c>
+      <c r="I33" s="9" t="n">
+        <v>885</v>
+      </c>
+      <c r="J33" s="9" t="n">
+        <v>555</v>
+      </c>
+      <c r="K33" s="8" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L33" s="8" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M33" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N33" s="10" t="inlineStr">
+        <is>
+          <t>Day 28: 28_prime_factors.py (Prime Factors of Number) | Extracted prime factors including repeated factors.</t>
+        </is>
+      </c>
+    </row>
     <row r="34" ht="22" customHeight="1"/>
     <row r="35" ht="22" customHeight="1"/>
     <row r="36" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 29 (10-Sep-2026): Practice 29 Perfect Number & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2158,7 +2158,60 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1"/>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>10-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>425</v>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>115</v>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>160</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I34" s="6" t="n">
+        <v>935</v>
+      </c>
+      <c r="J34" s="6" t="n">
+        <v>505</v>
+      </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N34" s="7" t="inlineStr">
+        <is>
+          <t>Day 29: 29_perfect_number.py (Check Perfect Number e.g. 28) | Checked proper divisor sum equality and searched range.</t>
+        </is>
+      </c>
+    </row>
     <row r="35" ht="22" customHeight="1"/>
     <row r="36" ht="22" customHeight="1"/>
     <row r="37" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 30 (11-Sep-2026): Practice 30 Armstrong Number & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2212,7 +2212,60 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="22" customHeight="1"/>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>11-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="n">
+        <v>420</v>
+      </c>
+      <c r="C35" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>180</v>
+      </c>
+      <c r="F35" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G35" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" s="9" t="n">
+        <v>145</v>
+      </c>
+      <c r="I35" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J35" s="9" t="n">
+        <v>440</v>
+      </c>
+      <c r="K35" s="8" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L35" s="8" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M35" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N35" s="10" t="inlineStr">
+        <is>
+          <t>Day 30: 30_armstrong_number.py (Armstrong Number Check) | Validated Armstrong numbers (e.g. 153, 370) under 1000.</t>
+        </is>
+      </c>
+    </row>
     <row r="36" ht="22" customHeight="1"/>
     <row r="37" ht="22" customHeight="1"/>
     <row r="38" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 31 (12-Sep-2026): Practice 31 Number Pattern & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2266,7 +2266,60 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="22" customHeight="1"/>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>12-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n">
+        <v>435</v>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>110</v>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>145</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>880</v>
+      </c>
+      <c r="J36" s="6" t="n">
+        <v>560</v>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N36" s="7" t="inlineStr">
+        <is>
+          <t>Day 31: 31_number_pattern.py (Number Pyramid Forward/Reverse) | Printed increasing and decreasing number pattern matrices.</t>
+        </is>
+      </c>
+    </row>
     <row r="37" ht="22" customHeight="1"/>
     <row r="38" ht="22" customHeight="1"/>
     <row r="39" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 32 (13-Sep-2026): Practice 32 Multiplication Grid & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2320,7 +2320,60 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="22" customHeight="1"/>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>13-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="n">
+        <v>430</v>
+      </c>
+      <c r="C37" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D37" s="9" t="n">
+        <v>115</v>
+      </c>
+      <c r="E37" s="9" t="n">
+        <v>155</v>
+      </c>
+      <c r="F37" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="I37" s="9" t="n">
+        <v>885</v>
+      </c>
+      <c r="J37" s="9" t="n">
+        <v>555</v>
+      </c>
+      <c r="K37" s="8" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L37" s="8" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M37" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N37" s="10" t="inlineStr">
+        <is>
+          <t>Day 32: 32_multiplication_grid.py (10x10 Multiplier Grid) | Rendered 10x10 multiplication table grid with nested loops.</t>
+        </is>
+      </c>
+    </row>
     <row r="38" ht="22" customHeight="1"/>
     <row r="39" ht="22" customHeight="1"/>
     <row r="40" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 33 (14-Sep-2026): Practice 33 Right Triangle Pattern & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2374,7 +2374,60 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="22" customHeight="1"/>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="n">
+        <v>460</v>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>125</v>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>140</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="I38" s="6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J38" s="6" t="n">
+        <v>440</v>
+      </c>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N38" s="7" t="inlineStr">
+        <is>
+          <t>Day 33: 33_right_triangle_pattern.py (Left &amp; Right Triangle) | Printed left-aligned and right-aligned star triangles.</t>
+        </is>
+      </c>
+    </row>
     <row r="39" ht="22" customHeight="1"/>
     <row r="40" ht="22" customHeight="1"/>
     <row r="41" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 34 (15-Sep-2026): Practice 34 Number Triangle & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N38"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2428,7 +2428,60 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="22" customHeight="1"/>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="n">
+        <v>465</v>
+      </c>
+      <c r="C39" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="D39" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="E39" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="F39" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G39" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="9" t="n">
+        <v>170</v>
+      </c>
+      <c r="I39" s="9" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J39" s="9" t="n">
+        <v>420</v>
+      </c>
+      <c r="K39" s="8" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L39" s="8" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M39" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N39" s="10" t="inlineStr">
+        <is>
+          <t>Day 34: 34_number_triangle.py (Repeated Number Triangle) | Printed repeated digit triangle (1, 22, 333, 4444, 55555).</t>
+        </is>
+      </c>
+    </row>
     <row r="40" ht="22" customHeight="1"/>
     <row r="41" ht="22" customHeight="1"/>
     <row r="42" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 35 (16-Sep-2026): Practice 35 Checkerboard Pattern & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2482,7 +2482,60 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="22" customHeight="1"/>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="n">
+        <v>435</v>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D40" s="6" t="n">
+        <v>110</v>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I40" s="6" t="n">
+        <v>880</v>
+      </c>
+      <c r="J40" s="6" t="n">
+        <v>560</v>
+      </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N40" s="7" t="inlineStr">
+        <is>
+          <t>Day 35: 35_checkerboard_pattern.py (N x N Checkerboard) | Created checkerboard pattern using (row + col) % 2 parity.</t>
+        </is>
+      </c>
+    </row>
     <row r="41" ht="22" customHeight="1"/>
     <row r="42" ht="22" customHeight="1"/>
     <row r="43" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 36 (17-Sep-2026): Practice 36 Atm Simulation & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2536,7 +2536,60 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="22" customHeight="1"/>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="n">
+        <v>435</v>
+      </c>
+      <c r="C41" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="D41" s="9" t="n">
+        <v>105</v>
+      </c>
+      <c r="E41" s="9" t="n">
+        <v>145</v>
+      </c>
+      <c r="F41" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G41" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" s="9" t="n">
+        <v>155</v>
+      </c>
+      <c r="I41" s="9" t="n">
+        <v>930</v>
+      </c>
+      <c r="J41" s="9" t="n">
+        <v>510</v>
+      </c>
+      <c r="K41" s="8" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L41" s="8" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M41" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N41" s="10" t="inlineStr">
+        <is>
+          <t>Day 36: 36_atm_simulation.py (ATM Menu-Driven Simulation) | Simulated ATM with balance check, deposits, and withdrawals.</t>
+        </is>
+      </c>
+    </row>
     <row r="42" ht="22" customHeight="1"/>
     <row r="43" ht="22" customHeight="1"/>
     <row r="44" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 37 (18-Sep-2026): Practice 37 Password Attempts & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2590,7 +2590,60 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="22" customHeight="1"/>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="n">
+        <v>425</v>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D42" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>160</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G42" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H42" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I42" s="6" t="n">
+        <v>990</v>
+      </c>
+      <c r="J42" s="6" t="n">
+        <v>450</v>
+      </c>
+      <c r="K42" s="5" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N42" s="7" t="inlineStr">
+        <is>
+          <t>Day 37: 37_password_attempts.py (Password Lockout 3 Tries) | Simulated 3-attempt password verification and account locking.</t>
+        </is>
+      </c>
+    </row>
     <row r="43" ht="22" customHeight="1"/>
     <row r="44" ht="22" customHeight="1"/>
     <row r="45" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 38 (19-Sep-2026): Practice 38 Number Guessing Game & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2644,7 +2644,60 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="22" customHeight="1"/>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>19-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="n">
+        <v>440</v>
+      </c>
+      <c r="C43" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="D43" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E43" s="9" t="n">
+        <v>140</v>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="9" t="n">
+        <v>160</v>
+      </c>
+      <c r="I43" s="9" t="n">
+        <v>880</v>
+      </c>
+      <c r="J43" s="9" t="n">
+        <v>560</v>
+      </c>
+      <c r="K43" s="8" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L43" s="8" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M43" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N43" s="10" t="inlineStr">
+        <is>
+          <t>Day 38: 38_number_guessing_game.py (Number Guessing Game) | Built guessing game giving Too High / Too Low hints.</t>
+        </is>
+      </c>
+    </row>
     <row r="44" ht="22" customHeight="1"/>
     <row r="45" ht="22" customHeight="1"/>
     <row r="46" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 39 (20-Sep-2026): Practice 39 Shopping Bill Discount & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2698,7 +2698,60 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="22" customHeight="1"/>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="n">
+        <v>435</v>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D44" s="6" t="n">
+        <v>105</v>
+      </c>
+      <c r="E44" s="6" t="n">
+        <v>135</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="6" t="n">
+        <v>155</v>
+      </c>
+      <c r="I44" s="6" t="n">
+        <v>865</v>
+      </c>
+      <c r="J44" s="6" t="n">
+        <v>575</v>
+      </c>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M44" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N44" s="7" t="inlineStr">
+        <is>
+          <t>Day 39: 39_shopping_bill_discount.py (Shopping Bill Discount) | Computed slab discounts (20%, 10%, 5%) on shopping bills.</t>
+        </is>
+      </c>
+    </row>
     <row r="45" ht="22" customHeight="1"/>
     <row r="46" ht="22" customHeight="1"/>
     <row r="47" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 40 (21-Sep-2026): Practice 40 Second Largest Number & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2752,7 +2752,60 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="22" customHeight="1"/>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="n">
+        <v>460</v>
+      </c>
+      <c r="C45" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D45" s="9" t="n">
+        <v>135</v>
+      </c>
+      <c r="E45" s="9" t="n">
+        <v>155</v>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G45" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" s="9" t="n">
+        <v>170</v>
+      </c>
+      <c r="I45" s="9" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J45" s="9" t="n">
+        <v>420</v>
+      </c>
+      <c r="K45" s="8" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L45" s="8" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M45" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N45" s="10" t="inlineStr">
+        <is>
+          <t>Day 40: 40_second_largest_number.py (Second Largest Number) | Found second-largest number without using sort() or max().</t>
+        </is>
+      </c>
+    </row>
     <row r="46" ht="22" customHeight="1"/>
     <row r="47" ht="22" customHeight="1"/>
     <row r="48" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 41 (22-Sep-2026): Practice 41 Frequency Of Digits & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2806,7 +2806,60 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="22" customHeight="1"/>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="n">
+        <v>465</v>
+      </c>
+      <c r="C46" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="D46" s="6" t="n">
+        <v>130</v>
+      </c>
+      <c r="E46" s="6" t="n">
+        <v>160</v>
+      </c>
+      <c r="F46" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" s="6" t="n">
+        <v>170</v>
+      </c>
+      <c r="I46" s="6" t="n">
+        <v>1030</v>
+      </c>
+      <c r="J46" s="6" t="n">
+        <v>410</v>
+      </c>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N46" s="7" t="inlineStr">
+        <is>
+          <t>Day 41: 41_frequency_of_digits.py (Digit Frequency Counter) | Counted occurrences of each digit 0-9 in large integer.</t>
+        </is>
+      </c>
+    </row>
     <row r="47" ht="22" customHeight="1"/>
     <row r="48" ht="22" customHeight="1"/>
     <row r="49" ht="22" customHeight="1"/>

</xml_diff>

<commit_message>
Day 42 (23-Sep-2026): Practice 42 Decimal To Binary & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2860,7 +2860,60 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="22" customHeight="1"/>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="n">
+        <v>430</v>
+      </c>
+      <c r="C47" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>125</v>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>165</v>
+      </c>
+      <c r="F47" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="I47" s="9" t="n">
+        <v>905</v>
+      </c>
+      <c r="J47" s="9" t="n">
+        <v>535</v>
+      </c>
+      <c r="K47" s="8" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L47" s="8" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M47" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N47" s="10" t="inlineStr">
+        <is>
+          <t>Day 42: 42_decimal_to_binary.py (Decimal to Binary Conversion) | Converted decimal number to binary string without bin().</t>
+        </is>
+      </c>
+    </row>
     <row r="48" ht="22" customHeight="1"/>
     <row r="49" ht="22" customHeight="1"/>
   </sheetData>

</xml_diff>

<commit_message>
Day 43 (24-Sep-2026): Practice 43 Strong Number & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2914,7 +2914,60 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="22" customHeight="1"/>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="n">
+        <v>430</v>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D48" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>170</v>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I48" s="6" t="n">
+        <v>960</v>
+      </c>
+      <c r="J48" s="6" t="n">
+        <v>480</v>
+      </c>
+      <c r="K48" s="5" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N48" s="7" t="inlineStr">
+        <is>
+          <t>Day 43: 43_strong_number.py (Strong Number e.g. 145) | Checked if number equals sum of factorials of its digits.</t>
+        </is>
+      </c>
+    </row>
     <row r="49" ht="22" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Day 44 (25-Sep-2026): Practice 44 Student Management System & update daily activity log
</commit_message>
<xml_diff>
--- a/12625876.xlsx
+++ b/12625876.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N48"/>
+  <dimension ref="A1:N49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2968,7 +2968,60 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="22" customHeight="1"/>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="n">
+        <v>420</v>
+      </c>
+      <c r="C49" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D49" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="E49" s="9" t="n">
+        <v>180</v>
+      </c>
+      <c r="F49" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G49" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H49" s="9" t="n">
+        <v>145</v>
+      </c>
+      <c r="I49" s="9" t="n">
+        <v>1010</v>
+      </c>
+      <c r="J49" s="9" t="n">
+        <v>430</v>
+      </c>
+      <c r="K49" s="8" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L49" s="8" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M49" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N49" s="10" t="inlineStr">
+        <is>
+          <t>Day 44: 44_student_management_system.py (Student Marks Analyzer) | Calculated 5-subject totals, percentages, class average, high/low.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:N3"/>

</xml_diff>